<commit_message>
Put the tie-detection camera and light bar on the front bumper
Both were carrying the placeholder "Underframe / center". The real location
is the front bumper, centre — which is what the audit tells someone walking
the machine where to look.

Fixtures re-cut against the corrected data, the Excel round-trip one through
Excel for Windows again, so an imported workbook does not silently revert the
location.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lib/master/__fixtures__/master-excel-roundtrip.xlsx
+++ b/src/lib/master/__fixtures__/master-excel-roundtrip.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bbmetalsky-my.sharepoint.com/personal/cotyc_bbrailtech_com/Documents/web-apps/Unit-Info (fleet)/src/lib/master/__fixtures__/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4BD0B6D-75E0-4BE3-A4E2-C0094CB5988E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3852D08-37F4-484A-BC13-3BB7B20EB8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8535" yWindow="465" windowWidth="11325" windowHeight="12690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0 Read Me" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
     <t>exported_at</t>
   </si>
   <si>
-    <t>2026-07-31T21:00:00.000Z</t>
+    <t>2026-08-03T00:00:00.000Z</t>
   </si>
   <si>
     <t>import_semantics</t>
@@ -415,7 +415,7 @@
     <t>Industrial camera</t>
   </si>
   <si>
-    <t>Underframe / center</t>
+    <t>Front bumper / center</t>
   </si>
   <si>
     <t>VT-4200-01</t>

</xml_diff>